<commit_message>
fix(sample): 501-a 复核修正——IB 示例参数网/存储网型号对齐 NVIDIA Quantum，example2 补 README
</commit_message>
<xml_diff>
--- a/example/128H100-IB/excel/hostname.xlsx
+++ b/example/128H100-IB/excel/hostname.xlsx
@@ -440,7 +440,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -547,7 +547,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>H3C S9827</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1226,7 +1226,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>H3C S9825-128B</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>H3C S9825-128B</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>H3C S9825-128B</t>
+          <t>NVIDIA Quantum QM9700</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>